<commit_message>
added function to ExcelWork
</commit_message>
<xml_diff>
--- a/src/main/resources/Opis_short.xlsx
+++ b/src/main/resources/Opis_short.xlsx
@@ -5,25 +5,25 @@
   <workbookPr codeName="ЭтаКнига" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IdeaProjects\ExcelWork\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IdeaProjects\LabSearch\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13872" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13875" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="оборудование" sheetId="4" r:id="rId1"/>
     <sheet name="комплектующие" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">комплектующие!$A$2:$H$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">комплектующие!$A$2:$H$7</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="37">
   <si>
     <t>№</t>
   </si>
@@ -142,6 +142,12 @@
   </si>
   <si>
     <t>BACK_SHELF</t>
+  </si>
+  <si>
+    <t>Провода</t>
+  </si>
+  <si>
+    <t>папа-папа</t>
   </si>
 </sst>
 </file>
@@ -676,13 +682,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>415636</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>51955</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>3082636</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>2520835</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1008,18 +1014,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Лист3"/>
   <dimension ref="A3:F8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.44140625" customWidth="1"/>
-    <col min="3" max="3" width="90.44140625" customWidth="1"/>
-    <col min="4" max="4" width="7.5546875" customWidth="1"/>
-    <col min="5" max="5" width="32.6640625" customWidth="1"/>
-    <col min="6" max="6" width="62.5546875" customWidth="1"/>
+    <col min="1" max="1" width="3.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" customWidth="1"/>
+    <col min="3" max="3" width="90.42578125" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" customWidth="1"/>
+    <col min="5" max="5" width="32.7109375" customWidth="1"/>
+    <col min="6" max="6" width="62.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="4" spans="1:6" ht="35.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:6" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>0</v>
       </c>
@@ -1039,7 +1045,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:6" s="4" customFormat="1" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" s="4" customFormat="1" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -1059,7 +1065,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:6" s="4" customFormat="1" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" s="4" customFormat="1" ht="150.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -1079,7 +1085,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:6" s="4" customFormat="1" ht="54.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" s="4" customFormat="1" ht="57" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -1099,7 +1105,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9"/>
       <c r="B8" s="27" t="s">
         <v>3</v>
@@ -1125,21 +1131,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Лист2"/>
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="200.1" customHeight="1" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="200.1" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.5546875" style="20" customWidth="1"/>
-    <col min="2" max="2" width="31.5546875" style="23" customWidth="1"/>
+    <col min="1" max="1" width="8.5703125" style="20" customWidth="1"/>
+    <col min="2" max="2" width="31.5703125" style="23" customWidth="1"/>
     <col min="3" max="3" width="90" style="24" customWidth="1"/>
-    <col min="4" max="4" width="9.5546875" style="23" customWidth="1"/>
-    <col min="5" max="5" width="50.6640625" style="13" customWidth="1"/>
-    <col min="6" max="6" width="80.33203125" style="14" customWidth="1"/>
-    <col min="7" max="7" width="38.6640625" style="13" customWidth="1"/>
-    <col min="8" max="16384" width="9.109375" style="13"/>
+    <col min="4" max="4" width="9.5703125" style="23" customWidth="1"/>
+    <col min="5" max="5" width="50.7109375" style="13" customWidth="1"/>
+    <col min="6" max="6" width="80.28515625" style="14" customWidth="1"/>
+    <col min="7" max="7" width="38.7109375" style="13" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>0</v>
       </c>
@@ -1162,7 +1168,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="200.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="21">
         <v>1</v>
       </c>
@@ -1183,7 +1189,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="200.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="22">
         <v>2</v>
       </c>
@@ -1204,7 +1210,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="200.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="21">
         <v>3</v>
       </c>
@@ -1225,31 +1231,43 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="200.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="22">
+    <row r="6" spans="1:7" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="21"/>
+      <c r="B6" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="25"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="17"/>
+    </row>
+    <row r="7" spans="1:7" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="22">
         <v>4</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B7" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="26" t="s">
+      <c r="C7" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="26">
+      <c r="D7" s="26">
         <v>18</v>
       </c>
-      <c r="E6" s="18"/>
-      <c r="F6" s="19" t="s">
+      <c r="E7" s="18"/>
+      <c r="F7" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="13" t="s">
+      <c r="G7" s="13" t="s">
         <v>34</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:H6"/>
+  <autoFilter ref="A2:H7"/>
   <hyperlinks>
-    <hyperlink ref="F6" r:id="rId1" display="http://amperka.ru/product/hc-06-bluetooth-module"/>
+    <hyperlink ref="F7" r:id="rId1" display="http://amperka.ru/product/hc-06-bluetooth-module"/>
     <hyperlink ref="F4" r:id="rId2" display="http://amperka.ru/product/troyka-bluetooth-hc-05"/>
     <hyperlink ref="F3" r:id="rId3" display="http://amperka.ru/product/3-wire-cable-extension"/>
     <hyperlink ref="F5" r:id="rId4"/>

</xml_diff>